<commit_message>
Extend MRPAM datasets with historical data 2021–2025 (issues #96–#99)
Added 2021–2023 historical data to all 7 MRPAM datasets by extracting
from cached monthly PDF reports. Updated charts to use temporal date axis
(year+month → datetime) for proper multi-year time series visualization.

Coverage by dataset:
- mrpam-coal-production: 2022–2025 (47 rows)
- mrpam-petroleum-production: 2021–2025 (52 rows)
- mrpam-mining-permits: 2023–2025 (748 rows)
- mrpam-commodity-prices: 2021–2025 (885 rows)
- mrpam-fuel-prices: 2023–2025 (781 rows)
- mrpam-petroleum-imports: 2021–2025 (466 rows)
- mrpam-budget-revenue: 2023–2025 (248 rows)

Note: Some years/datasets excluded due to PDF format changes that caused
extraction errors (2021–2022 budget revenue, fuel prices; 2022 mining permits).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/mrpam-coal-production.xlsx
+++ b/data.mn/public/datasets/mrpam-coal-production.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,13 +26,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,8 +56,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,31 +426,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>production_kt</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>sales_kt</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>export_kt</t>
         </is>
@@ -446,205 +465,800 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>5880.8</v>
+        <v>2163.5</v>
       </c>
       <c r="D2" t="n">
-        <v>4693.5</v>
+        <v>1636.2</v>
       </c>
       <c r="E2" t="n">
-        <v>3406.2</v>
+        <v>443.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>7347.8</v>
+        <v>1626.4</v>
       </c>
       <c r="D3" t="n">
-        <v>5456.9</v>
+        <v>1571.1</v>
       </c>
       <c r="E3" t="n">
-        <v>4504.8</v>
+        <v>503.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>7987.8</v>
+        <v>2344.6</v>
       </c>
       <c r="D4" t="n">
-        <v>4921.5</v>
+        <v>1427.2</v>
       </c>
       <c r="E4" t="n">
-        <v>3897</v>
+        <v>680</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>8718.299999999999</v>
+        <v>1923.6</v>
       </c>
       <c r="D5" t="n">
-        <v>7829.5</v>
+        <v>1433.9</v>
       </c>
       <c r="E5" t="n">
-        <v>7091.4</v>
+        <v>832.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>9147.200000000001</v>
+        <v>2129.5</v>
       </c>
       <c r="D6" t="n">
-        <v>7025.7</v>
+        <v>2287.1</v>
       </c>
       <c r="E6" t="n">
-        <v>6282.9</v>
+        <v>1757.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>6626.1</v>
+        <v>2304.8</v>
       </c>
       <c r="D7" t="n">
-        <v>5289.2</v>
+        <v>2936.1</v>
       </c>
       <c r="E7" t="n">
-        <v>4910.1</v>
+        <v>2434.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>7981.4</v>
+        <v>3601.9</v>
       </c>
       <c r="D8" t="n">
-        <v>7315.1</v>
+        <v>3821.1</v>
       </c>
       <c r="E8" t="n">
-        <v>6672</v>
+        <v>3083.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" t="n">
-        <v>7627.9</v>
+        <v>4249.4</v>
       </c>
       <c r="D9" t="n">
-        <v>6783.5</v>
+        <v>4941.4</v>
       </c>
       <c r="E9" t="n">
-        <v>6116.6</v>
+        <v>3849.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>10130.1</v>
+        <v>5128.2</v>
       </c>
       <c r="D10" t="n">
-        <v>10105.3</v>
+        <v>5295.3</v>
       </c>
       <c r="E10" t="n">
-        <v>9100.4</v>
+        <v>3954.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" t="n">
-        <v>10165.9</v>
+        <v>5417.9</v>
       </c>
       <c r="D11" t="n">
-        <v>8382.5</v>
+        <v>5530.4</v>
       </c>
       <c r="E11" t="n">
-        <v>7065</v>
+        <v>4181.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" t="n">
-        <v>11089.8</v>
+        <v>6403.4</v>
       </c>
       <c r="D12" t="n">
-        <v>9459.200000000001</v>
+        <v>6294</v>
       </c>
       <c r="E12" t="n">
-        <v>8320.799999999999</v>
+        <v>4844.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>5579.1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5759.1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4282.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4777</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5453.8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4204.4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>6592.1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6653.2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5430.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5791.2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5569</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4611</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5947.7</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4894.6</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4152</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" t="n">
+        <v>6195.1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4779.4</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4113.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B19" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" t="n">
+        <v>5720.8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>5827.8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5098.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="n">
+        <v>7908.8</v>
+      </c>
+      <c r="D20" t="n">
+        <v>7525</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6744.3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B21" t="n">
+        <v>9</v>
+      </c>
+      <c r="C21" t="n">
+        <v>8530.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>7706.1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6882.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B22" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" t="n">
+        <v>9090.200000000001</v>
+      </c>
+      <c r="D22" t="n">
+        <v>8022.1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>6712.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B23" t="n">
+        <v>11</v>
+      </c>
+      <c r="C23" t="n">
+        <v>24203.6</v>
+      </c>
+      <c r="D23" t="n">
+        <v>38310.3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>38481.8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B24" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C24" t="n">
+        <v>8452</v>
+      </c>
+      <c r="D24" t="n">
+        <v>8372.4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6667.3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>7072.2</v>
+      </c>
+      <c r="D25" t="n">
+        <v>6749</v>
+      </c>
+      <c r="E25" t="n">
+        <v>5385.6</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>7004.3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5714.7</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4468.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8337.299999999999</v>
+      </c>
+      <c r="D27" t="n">
+        <v>7247</v>
+      </c>
+      <c r="E27" t="n">
+        <v>6003.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>9171.700000000001</v>
+      </c>
+      <c r="D28" t="n">
+        <v>7512</v>
+      </c>
+      <c r="E28" t="n">
+        <v>6470.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" t="n">
+        <v>9148.1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>7542.4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>6649.8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B30" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" t="n">
+        <v>8883.1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>7814.4</v>
+      </c>
+      <c r="E30" t="n">
+        <v>7010.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B31" t="n">
+        <v>7</v>
+      </c>
+      <c r="C31" t="n">
+        <v>8629.9</v>
+      </c>
+      <c r="D31" t="n">
+        <v>7514</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6892.7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C32" t="n">
+        <v>8701.4</v>
+      </c>
+      <c r="D32" t="n">
+        <v>7554.7</v>
+      </c>
+      <c r="E32" t="n">
+        <v>6710.9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B33" t="n">
+        <v>9</v>
+      </c>
+      <c r="C33" t="n">
+        <v>9363</v>
+      </c>
+      <c r="D33" t="n">
+        <v>7068.6</v>
+      </c>
+      <c r="E33" t="n">
+        <v>6075.4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B34" t="n">
+        <v>10</v>
+      </c>
+      <c r="C34" t="n">
+        <v>10268.7</v>
+      </c>
+      <c r="D34" t="n">
+        <v>8044.3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>6828.7</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B35" t="n">
+        <v>11</v>
+      </c>
+      <c r="C35" t="n">
+        <v>10474.4</v>
+      </c>
+      <c r="D35" t="n">
+        <v>6997.9</v>
+      </c>
+      <c r="E35" t="n">
+        <v>5601.5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B36" t="n">
+        <v>12</v>
+      </c>
+      <c r="C36" t="n">
+        <v>9486.799999999999</v>
+      </c>
+      <c r="D36" t="n">
+        <v>7860.9</v>
+      </c>
+      <c r="E36" t="n">
+        <v>6312.8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>5880.8</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4693.5</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3406.2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="n">
+        <v>7347.8</v>
+      </c>
+      <c r="D38" t="n">
+        <v>5456.9</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4504.8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="n">
+        <v>7987.8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>4921.5</v>
+      </c>
+      <c r="E39" t="n">
+        <v>3897</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n">
+        <v>8718.299999999999</v>
+      </c>
+      <c r="D40" t="n">
+        <v>7829.5</v>
+      </c>
+      <c r="E40" t="n">
+        <v>7091.4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" t="n">
+        <v>9147.200000000001</v>
+      </c>
+      <c r="D41" t="n">
+        <v>7025.7</v>
+      </c>
+      <c r="E41" t="n">
+        <v>6282.9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" t="n">
+        <v>6626.1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5289.2</v>
+      </c>
+      <c r="E42" t="n">
+        <v>4910.1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B43" t="n">
+        <v>7</v>
+      </c>
+      <c r="C43" t="n">
+        <v>7981.4</v>
+      </c>
+      <c r="D43" t="n">
+        <v>7315.1</v>
+      </c>
+      <c r="E43" t="n">
+        <v>6672</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" t="n">
+        <v>7627.9</v>
+      </c>
+      <c r="D44" t="n">
+        <v>6783.5</v>
+      </c>
+      <c r="E44" t="n">
+        <v>6116.6</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B45" t="n">
+        <v>9</v>
+      </c>
+      <c r="C45" t="n">
+        <v>10130.1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>10105.3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>9100.4</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B46" t="n">
+        <v>10</v>
+      </c>
+      <c r="C46" t="n">
+        <v>10165.9</v>
+      </c>
+      <c r="D46" t="n">
+        <v>8382.5</v>
+      </c>
+      <c r="E46" t="n">
+        <v>7065</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B47" t="n">
+        <v>11</v>
+      </c>
+      <c r="C47" t="n">
+        <v>11089.8</v>
+      </c>
+      <c r="D47" t="n">
+        <v>9459.200000000001</v>
+      </c>
+      <c r="E47" t="n">
+        <v>8320.799999999999</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B48" t="n">
+        <v>12</v>
+      </c>
+      <c r="C48" t="n">
         <v>11350.5</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D48" t="n">
         <v>10503.8</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E48" t="n">
         <v>9115.700000000001</v>
       </c>
     </row>
@@ -659,31 +1273,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>он</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>сар</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>олборлолт_мян_тн</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>борлуулалт_мян_тн</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>экспорт_мян_тн</t>
         </is>
@@ -691,205 +1312,800 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>5880.8</v>
+        <v>2163.5</v>
       </c>
       <c r="D2" t="n">
-        <v>4693.5</v>
+        <v>1636.2</v>
       </c>
       <c r="E2" t="n">
-        <v>3406.2</v>
+        <v>443.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>7347.8</v>
+        <v>1626.4</v>
       </c>
       <c r="D3" t="n">
-        <v>5456.9</v>
+        <v>1571.1</v>
       </c>
       <c r="E3" t="n">
-        <v>4504.8</v>
+        <v>503.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>7987.8</v>
+        <v>2344.6</v>
       </c>
       <c r="D4" t="n">
-        <v>4921.5</v>
+        <v>1427.2</v>
       </c>
       <c r="E4" t="n">
-        <v>3897</v>
+        <v>680</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>8718.299999999999</v>
+        <v>1923.6</v>
       </c>
       <c r="D5" t="n">
-        <v>7829.5</v>
+        <v>1433.9</v>
       </c>
       <c r="E5" t="n">
-        <v>7091.4</v>
+        <v>832.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>9147.200000000001</v>
+        <v>2129.5</v>
       </c>
       <c r="D6" t="n">
-        <v>7025.7</v>
+        <v>2287.1</v>
       </c>
       <c r="E6" t="n">
-        <v>6282.9</v>
+        <v>1757.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>6626.1</v>
+        <v>2304.8</v>
       </c>
       <c r="D7" t="n">
-        <v>5289.2</v>
+        <v>2936.1</v>
       </c>
       <c r="E7" t="n">
-        <v>4910.1</v>
+        <v>2434.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>7981.4</v>
+        <v>3601.9</v>
       </c>
       <c r="D8" t="n">
-        <v>7315.1</v>
+        <v>3821.1</v>
       </c>
       <c r="E8" t="n">
-        <v>6672</v>
+        <v>3083.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" t="n">
-        <v>7627.9</v>
+        <v>4249.4</v>
       </c>
       <c r="D9" t="n">
-        <v>6783.5</v>
+        <v>4941.4</v>
       </c>
       <c r="E9" t="n">
-        <v>6116.6</v>
+        <v>3849.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>10130.1</v>
+        <v>5128.2</v>
       </c>
       <c r="D10" t="n">
-        <v>10105.3</v>
+        <v>5295.3</v>
       </c>
       <c r="E10" t="n">
-        <v>9100.4</v>
+        <v>3954.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" t="n">
-        <v>10165.9</v>
+        <v>5417.9</v>
       </c>
       <c r="D11" t="n">
-        <v>8382.5</v>
+        <v>5530.4</v>
       </c>
       <c r="E11" t="n">
-        <v>7065</v>
+        <v>4181.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" t="n">
-        <v>11089.8</v>
+        <v>6403.4</v>
       </c>
       <c r="D12" t="n">
-        <v>9459.200000000001</v>
+        <v>6294</v>
       </c>
       <c r="E12" t="n">
-        <v>8320.799999999999</v>
+        <v>4844.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>5579.1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5759.1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4282.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4777</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5453.8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4204.4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>6592.1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6653.2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5430.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5791.2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5569</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4611</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5947.7</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4894.6</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4152</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" t="n">
+        <v>6195.1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4779.4</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4113.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B19" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" t="n">
+        <v>5720.8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>5827.8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5098.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="n">
+        <v>7908.8</v>
+      </c>
+      <c r="D20" t="n">
+        <v>7525</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6744.3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B21" t="n">
+        <v>9</v>
+      </c>
+      <c r="C21" t="n">
+        <v>8530.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>7706.1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6882.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B22" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" t="n">
+        <v>9090.200000000001</v>
+      </c>
+      <c r="D22" t="n">
+        <v>8022.1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>6712.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B23" t="n">
+        <v>11</v>
+      </c>
+      <c r="C23" t="n">
+        <v>24203.6</v>
+      </c>
+      <c r="D23" t="n">
+        <v>38310.3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>38481.8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B24" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C24" t="n">
+        <v>8452</v>
+      </c>
+      <c r="D24" t="n">
+        <v>8372.4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6667.3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>7072.2</v>
+      </c>
+      <c r="D25" t="n">
+        <v>6749</v>
+      </c>
+      <c r="E25" t="n">
+        <v>5385.6</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>7004.3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5714.7</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4468.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8337.299999999999</v>
+      </c>
+      <c r="D27" t="n">
+        <v>7247</v>
+      </c>
+      <c r="E27" t="n">
+        <v>6003.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>9171.700000000001</v>
+      </c>
+      <c r="D28" t="n">
+        <v>7512</v>
+      </c>
+      <c r="E28" t="n">
+        <v>6470.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" t="n">
+        <v>9148.1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>7542.4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>6649.8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B30" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" t="n">
+        <v>8883.1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>7814.4</v>
+      </c>
+      <c r="E30" t="n">
+        <v>7010.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B31" t="n">
+        <v>7</v>
+      </c>
+      <c r="C31" t="n">
+        <v>8629.9</v>
+      </c>
+      <c r="D31" t="n">
+        <v>7514</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6892.7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C32" t="n">
+        <v>8701.4</v>
+      </c>
+      <c r="D32" t="n">
+        <v>7554.7</v>
+      </c>
+      <c r="E32" t="n">
+        <v>6710.9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B33" t="n">
+        <v>9</v>
+      </c>
+      <c r="C33" t="n">
+        <v>9363</v>
+      </c>
+      <c r="D33" t="n">
+        <v>7068.6</v>
+      </c>
+      <c r="E33" t="n">
+        <v>6075.4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B34" t="n">
+        <v>10</v>
+      </c>
+      <c r="C34" t="n">
+        <v>10268.7</v>
+      </c>
+      <c r="D34" t="n">
+        <v>8044.3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>6828.7</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B35" t="n">
+        <v>11</v>
+      </c>
+      <c r="C35" t="n">
+        <v>10474.4</v>
+      </c>
+      <c r="D35" t="n">
+        <v>6997.9</v>
+      </c>
+      <c r="E35" t="n">
+        <v>5601.5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B36" t="n">
+        <v>12</v>
+      </c>
+      <c r="C36" t="n">
+        <v>9486.799999999999</v>
+      </c>
+      <c r="D36" t="n">
+        <v>7860.9</v>
+      </c>
+      <c r="E36" t="n">
+        <v>6312.8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>5880.8</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4693.5</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3406.2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="n">
+        <v>7347.8</v>
+      </c>
+      <c r="D38" t="n">
+        <v>5456.9</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4504.8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="n">
+        <v>7987.8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>4921.5</v>
+      </c>
+      <c r="E39" t="n">
+        <v>3897</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n">
+        <v>8718.299999999999</v>
+      </c>
+      <c r="D40" t="n">
+        <v>7829.5</v>
+      </c>
+      <c r="E40" t="n">
+        <v>7091.4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" t="n">
+        <v>9147.200000000001</v>
+      </c>
+      <c r="D41" t="n">
+        <v>7025.7</v>
+      </c>
+      <c r="E41" t="n">
+        <v>6282.9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" t="n">
+        <v>6626.1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5289.2</v>
+      </c>
+      <c r="E42" t="n">
+        <v>4910.1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B43" t="n">
+        <v>7</v>
+      </c>
+      <c r="C43" t="n">
+        <v>7981.4</v>
+      </c>
+      <c r="D43" t="n">
+        <v>7315.1</v>
+      </c>
+      <c r="E43" t="n">
+        <v>6672</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" t="n">
+        <v>7627.9</v>
+      </c>
+      <c r="D44" t="n">
+        <v>6783.5</v>
+      </c>
+      <c r="E44" t="n">
+        <v>6116.6</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B45" t="n">
+        <v>9</v>
+      </c>
+      <c r="C45" t="n">
+        <v>10130.1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>10105.3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>9100.4</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B46" t="n">
+        <v>10</v>
+      </c>
+      <c r="C46" t="n">
+        <v>10165.9</v>
+      </c>
+      <c r="D46" t="n">
+        <v>8382.5</v>
+      </c>
+      <c r="E46" t="n">
+        <v>7065</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B47" t="n">
+        <v>11</v>
+      </c>
+      <c r="C47" t="n">
+        <v>11089.8</v>
+      </c>
+      <c r="D47" t="n">
+        <v>9459.200000000001</v>
+      </c>
+      <c r="E47" t="n">
+        <v>8320.799999999999</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B48" t="n">
+        <v>12</v>
+      </c>
+      <c r="C48" t="n">
         <v>11350.5</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D48" t="n">
         <v>10503.8</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E48" t="n">
         <v>9115.700000000001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MRPAM: Fill 2021 gap in coal-production dataset (from PR #105)
Salvaged the coal-production portion of PR #105 — the only dataset with
matching schema between main and the intern's branch. Appends 12 rows
for 2021 monthly values (production_kt, sales_kt, export_kt).

- Unioned main + PR #105 CSVs on (year, month), dedup-kept main's version
- Regenerated wide-form XLSX (annual sums by metric)
- Updated EN/MN MDX title and excerpt: 2022–2025 → 2021–2025

Did NOT merge the PR's fuel-prices, budget-revenue, or mining-permits
changes — those three datasets have schema divergence vs. current main
(column renames, missing pct_of_plan/хувь, province transliterations
like Bayan-Ulgii vs Bayan-Ölgii). The intern should redo those against
current main.

Closes the 2021 gap noted in e52f16b7 for coal-production only.

Co-Authored-By: OkuOrgil3757 <m.enkh-orgil@letumongolia.com>
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/mrpam-coal-production.xlsx
+++ b/data.mn/public/datasets/mrpam-coal-production.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EN" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MN" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EN" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="MN" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,20 +30,15 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -51,14 +46,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -425,15 +426,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -442,15 +436,18 @@
         </is>
       </c>
       <c r="B1" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C1" s="1" t="n">
         <v>2022</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="D1" s="1" t="n">
         <v>2023</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="E1" s="1" t="n">
         <v>2024</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="F1" s="1" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -461,15 +458,18 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>32317.6</v>
+      </c>
+      <c r="C2" t="n">
         <v>37293.2</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>98788.10000000001</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>106540.9</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>104053.6</v>
       </c>
     </row>
@@ -480,15 +480,18 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>26741.6</v>
+      </c>
+      <c r="C3" t="n">
         <v>37173.8</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>108872.8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>87619.89999999999</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>87765.7</v>
       </c>
     </row>
@@ -499,15 +502,18 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>15932.9</v>
+      </c>
+      <c r="C4" t="n">
         <v>26563.5</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>97380.3</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>74409.2</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>76482.89999999999</v>
       </c>
     </row>
@@ -522,15 +528,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -539,15 +538,18 @@
         </is>
       </c>
       <c r="B1" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C1" s="1" t="n">
         <v>2022</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="D1" s="1" t="n">
         <v>2023</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="E1" s="1" t="n">
         <v>2024</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="F1" s="1" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -558,15 +560,18 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>32317.6</v>
+      </c>
+      <c r="C2" t="n">
         <v>37293.2</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>98788.10000000001</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>106540.9</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>104053.6</v>
       </c>
     </row>
@@ -577,15 +582,18 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>26741.6</v>
+      </c>
+      <c r="C3" t="n">
         <v>37173.8</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>108872.8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>87619.89999999999</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>87765.7</v>
       </c>
     </row>
@@ -596,15 +604,18 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>15932.9</v>
+      </c>
+      <c r="C4" t="n">
         <v>26563.5</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>97380.3</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>74409.2</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>76482.89999999999</v>
       </c>
     </row>

</xml_diff>